<commit_message>
GEO Monitor: adaptado a la plantilla definitiva (pestañas prompts y resultados)
Columnas de resultados: estado (ok, sin_overview, error), menciona_bcp,
posicion_bcp, marcas_mencionadas, citado_bcp. Prompts usa fecha_creacion.
El Sheet está creado en Drive y su ID publicado en n8n.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U1VzVvGvVZYDf9tBgWaAmF
</commit_message>
<xml_diff>
--- a/automatizacion/geo-monitor/plantilla-geo-monitor.xlsx
+++ b/automatizacion/geo-monitor/plantilla-geo-monitor.xlsx
@@ -7,9 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompts" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Léeme" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="prompts" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="resultados" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,10 +29,6 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="14"/>
     </font>
   </fonts>
   <fills count="3">
@@ -61,10 +56,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,16 +424,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -470,99 +463,88 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>creado</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>actualizado</t>
+          <t>fecha_creacion</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>p_ahorro1</t>
+          <t>p001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Cuentas de ahorro</t>
+          <t>Marca</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>¿Cuál es el mejor banco del Perú para abrir una cuenta de ahorros?</t>
+          <t>¿Cuál es el mejor banco del Perú?</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Producto</t>
-        </is>
-      </c>
-      <c r="E2" t="b">
-        <v>1</v>
+          <t>Reputación</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-10-20T12:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2026-10-20T12:00:00.000Z</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>p_ahorro2</t>
+          <t>p002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cuentas de ahorro</t>
+          <t>Marca</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>¿Qué banco en Perú da la mejor tasa para un depósito a plazo fijo?</t>
+          <t>¿Cuál es el banco más seguro y confiable del Perú?</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Producto</t>
-        </is>
-      </c>
-      <c r="E3" t="b">
-        <v>1</v>
+          <t>Reputación</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-10-20T12:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>2026-10-20T12:00:00.000Z</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>p_tarjeta1</t>
+          <t>p003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Tarjetas de crédito</t>
+          <t>Cuentas</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>¿Qué tarjeta de crédito me conviene en Perú para acumular millas?</t>
+          <t>¿Qué banco me recomiendas para abrir una cuenta de ahorros en Perú?</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -570,34 +552,31 @@
           <t>Producto</t>
         </is>
       </c>
-      <c r="E4" t="b">
-        <v>1</v>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-10-20T12:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>2026-10-20T12:00:00.000Z</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>p_tarjeta2</t>
+          <t>p004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Tarjetas de crédito</t>
+          <t>Tarjetas</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>¿Qué banco peruano cobra menos comisiones en su tarjeta de crédito?</t>
+          <t>¿Cuál es la mejor tarjeta de crédito en Perú para acumular millas?</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -605,87 +584,78 @@
           <t>Producto</t>
         </is>
       </c>
-      <c r="E5" t="b">
-        <v>1</v>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-10-20T12:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2026-10-20T12:00:00.000Z</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>p_digital1</t>
+          <t>p005</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Banca digital</t>
+          <t>Hipotecario</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>¿Cuál es la mejor app de banca móvil en Perú?</t>
+          <t>¿Qué banco ofrece el mejor crédito hipotecario en Lima?</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Digital</t>
-        </is>
-      </c>
-      <c r="E6" t="b">
-        <v>1</v>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-10-20T12:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>2026-10-20T12:00:00.000Z</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>p_reputa1</t>
+          <t>p006</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Reputación</t>
+          <t>Digital</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>¿Cuál es el banco más confiable y seguro del Perú?</t>
+          <t>¿Cuál es la mejor app bancaria del Perú?</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Reputación</t>
-        </is>
-      </c>
-      <c r="E7" t="b">
-        <v>1</v>
+          <t>Digital</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-10-20T12:00:00.000Z</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>2026-10-20T12:00:00.000Z</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -703,23 +673,23 @@
   <dimension ref="A1:Q1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="30" customWidth="1" min="14" max="14"/>
-    <col width="40" customWidth="1" min="15" max="15"/>
-    <col width="80" customWidth="1" min="16" max="16"/>
-    <col width="30" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -750,14 +720,14 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>categoria</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>prompt</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>categoria</t>
-        </is>
-      </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>motor</t>
@@ -765,17 +735,17 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>disponible</t>
+          <t>estado</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>menciona</t>
+          <t>menciona_bcp</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>posicion</t>
+          <t>posicion_bcp</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
@@ -785,127 +755,27 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>citado</t>
+          <t>marcas_mencionadas</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>marcas</t>
+          <t>fuentes</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>fuentes</t>
+          <t>citado_bcp</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
           <t>respuesta</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>error</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>GEO Monitor — cómo usar esta hoja</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Prompts: lo que se pregunta a cada motor. Se edita desde el front (/geo-prompts-save) o a mano.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  · id: único y sin espacios. Si agregas filas a mano, inventa uno (p_algo).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  · activo: TRUE entra en la corrida diaria; FALSE no. «Eliminar» desde el front lo pone en FALSE.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  · categoria: Reputación, Producto, Digital u Otra.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Resultados: lo escribe el workflow, una fila por prompt y motor en cada corrida. No la edites.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  · disponible: el motor devolvió respuesta (en AI Overview: Google mostró un AI Overview).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  · posicion: orden en que aparece BCP entre las marcas mencionadas (1 = la primera).</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  · sentimiento: de -1 a 1, por diccionario de palabras alrededor de cada mención de BCP.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  · error: si el motor falló (saldo, modelo, límite). Esas filas no cuentan en el dashboard.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>No cambies los nombres de las pestañas ni de las columnas de la fila 1: el workflow los usa.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
GEO Monitor: el front lee los datos en vivo de n8n
Nuevo endpoint geo-monitor-data con la forma DATA.monitor del front «BCP ·
Monitor de Visibilidad en IA», que ahora vive en front/ con un loader.js que
lo carga antes de arrancar las vistas y vuelve a la demo si n8n no responde.

En la corrida: el Analista IA pasa a Claude Haiku (GEMINI BCP sin saldo),
cuenta menciones para el SOV por respuesta y normaliza los nombres de los
bancos. dominioDe ya no usa URL, que el sandbox de n8n no trae y dejaba las
fuentes vacías. La segunda llamada de AI Overview usa locations.json en vez
de account.json, que devolvía la API key. Si el Analista falla, la fila va
como error y no como «no menciona».

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U1VzVvGvVZYDf9tBgWaAmF
</commit_message>
<xml_diff>
--- a/automatizacion/geo-monitor/plantilla-geo-monitor.xlsx
+++ b/automatizacion/geo-monitor/plantilla-geo-monitor.xlsx
@@ -670,7 +670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:S1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -778,6 +778,16 @@
           <t>respuesta</t>
         </is>
       </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>n_menciones_bcp</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>n_menciones_bancos</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>